<commit_message>
ajuste modelos datos y procesos subyacentes
</commit_message>
<xml_diff>
--- a/MODELO_DATOS_COTIZADOR.xlsx
+++ b/MODELO_DATOS_COTIZADOR.xlsx
@@ -285,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -447,6 +447,12 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5659,7 +5665,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5773,29 +5779,29 @@
       <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>unidad</t>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>proyecto</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>uq_unidad_por_proyecto</t>
+          <t>idx_proyecto_cascada</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>id_proyecto, tipo_unidad, numero_unidad</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Único PARCIAL WHERE numero_unidad IS NOT NULL</t>
+          <t>comuna, tipo_entrega, id_inmobiliaria, activo  WHERE activo=1</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Integridad: no duplicados reales. Permite múltiples NULLs</t>
+          <t>Dropdown en cascada: Comuna → Entrega → Inmobiliaria → Proyecto</t>
         </is>
       </c>
     </row>
@@ -5810,22 +5816,22 @@
       </c>
       <c r="C6" s="55" t="inlineStr">
         <is>
-          <t>idx_unidad_proyecto</t>
+          <t>uq_unidad_por_proyecto</t>
         </is>
       </c>
       <c r="D6" s="55" t="inlineStr">
         <is>
-          <t>id_proyecto</t>
-        </is>
-      </c>
-      <c r="E6" s="56" t="inlineStr">
-        <is>
-          <t>Normal</t>
+          <t>id_proyecto, tipo_unidad, numero_unidad</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>Único PARCIAL WHERE numero_unidad IS NOT NULL</t>
         </is>
       </c>
       <c r="F6" s="55" t="inlineStr">
         <is>
-          <t>Lookup FK</t>
+          <t>Integridad: no duplicados reales. Permite múltiples NULLs</t>
         </is>
       </c>
     </row>
@@ -5840,12 +5846,12 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>idx_unidad_disponibles</t>
+          <t>idx_unidad_proyecto</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>id_proyecto, estado_stock, tipo_unidad</t>
+          <t>id_proyecto</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -5855,7 +5861,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Filtro principal del cotizador (unidades disponibles)</t>
+          <t>Lookup FK</t>
         </is>
       </c>
     </row>
@@ -5870,12 +5876,12 @@
       </c>
       <c r="C8" s="55" t="inlineStr">
         <is>
-          <t>idx_unidad_numero</t>
+          <t>idx_unidad_disponibles</t>
         </is>
       </c>
       <c r="D8" s="55" t="inlineStr">
         <is>
-          <t>numero_unidad</t>
+          <t>id_proyecto, estado_stock, tipo_unidad</t>
         </is>
       </c>
       <c r="E8" s="56" t="inlineStr">
@@ -5885,7 +5891,7 @@
       </c>
       <c r="F8" s="55" t="inlineStr">
         <is>
-          <t>Selección por número de unidad en la UI</t>
+          <t>Filtro principal del cotizador (unidades disponibles)</t>
         </is>
       </c>
     </row>
@@ -5900,12 +5906,12 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>idx_unidad_precio</t>
+          <t>idx_unidad_numero</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>id_proyecto, precio_lista_uf</t>
+          <t>numero_unidad</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -5915,7 +5921,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Ordenamiento por precio</t>
+          <t>Selección por número de unidad en la UI</t>
         </is>
       </c>
     </row>
@@ -5930,12 +5936,12 @@
       </c>
       <c r="C10" s="55" t="inlineStr">
         <is>
-          <t>idx_unidad_condicion</t>
+          <t>idx_unidad_precio</t>
         </is>
       </c>
       <c r="D10" s="55" t="inlineStr">
         <is>
-          <t>id_proyecto, tipo_unidad, programa</t>
+          <t>id_proyecto, precio_lista_uf</t>
         </is>
       </c>
       <c r="E10" s="56" t="inlineStr">
@@ -5945,7 +5951,7 @@
       </c>
       <c r="F10" s="55" t="inlineStr">
         <is>
-          <t>JOIN con condicion_comercial</t>
+          <t>Ordenamiento por precio</t>
         </is>
       </c>
     </row>
@@ -5953,14 +5959,14 @@
       <c r="A11" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>condicion_comercial</t>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>unidad</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>uq_condicion</t>
+          <t>idx_unidad_condicion</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -5968,14 +5974,14 @@
           <t>id_proyecto, tipo_unidad, programa</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Único</t>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Normal</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Clave natural: una condición por proyecto + tipo + programa</t>
+          <t>JOIN con condicion_comercial</t>
         </is>
       </c>
     </row>
@@ -5990,22 +5996,22 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>idx_condicion_proyecto</t>
+          <t>uq_condicion</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>id_proyecto, activo</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>Normal</t>
+          <t>id_proyecto, tipo_unidad, programa</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Único</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Filtro por proyecto</t>
+          <t>Clave natural: una condición por proyecto + tipo + programa</t>
         </is>
       </c>
     </row>
@@ -6020,52 +6026,52 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
+          <t>idx_condicion_proyecto</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>id_proyecto, activo</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Filtro por proyecto</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>condicion_comercial</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
           <t>idx_condicion_join</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>id_proyecto, tipo_unidad, programa  WHERE activo=1</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>Parcial activos</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>JOIN del cotizador solo con condiciones activas</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="30" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>bien_conjunto</t>
-        </is>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>idx_bc_principal</t>
-        </is>
-      </c>
-      <c r="D14" s="40" t="inlineStr">
-        <is>
-          <t>id_unidad_principal</t>
-        </is>
-      </c>
-      <c r="E14" s="39" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="F14" s="40" t="inlineStr">
-        <is>
-          <t>Lookup de bienes del departamento</t>
         </is>
       </c>
     </row>
@@ -6080,52 +6086,52 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
+          <t>idx_bc_principal</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>id_unidad_principal</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>Lookup de bienes del departamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="30" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>bien_conjunto</t>
+        </is>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
           <t>idx_bc_asociada</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="40" t="inlineStr">
         <is>
           <t>id_unidad_asociada</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="E16" s="39" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F16" s="40" t="inlineStr">
         <is>
           <t>Lookup del departamento al que pertenece un bien</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" s="19" t="inlineStr">
-        <is>
-          <t>uf_valor</t>
-        </is>
-      </c>
-      <c r="C16" s="21" t="inlineStr">
-        <is>
-          <t>idx_uf_fecha_desc</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>fecha DESC</t>
-        </is>
-      </c>
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="F16" s="21" t="inlineStr">
-        <is>
-          <t>Lookup eficiente del valor UF más reciente (MAX fecha)</t>
         </is>
       </c>
     </row>
@@ -6133,59 +6139,59 @@
       <c r="A17" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>uf_valor</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>idx_uf_fecha_desc</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>fecha DESC</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Lookup eficiente del valor UF más reciente (MAX fecha)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>parametro_cotizador</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="57" t="inlineStr">
         <is>
           <t>idx_parametro_categoria</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D18" s="57" t="inlineStr">
         <is>
           <t>categoria, activo</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="58" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="F18" s="57" t="inlineStr">
         <is>
           <t>Carga de dropdowns de la UI</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="23" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="24" t="inlineStr">
-        <is>
-          <t>cotizacion</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="inlineStr">
-        <is>
-          <t>idx_cotizacion_unidad</t>
-        </is>
-      </c>
-      <c r="D18" s="26" t="inlineStr">
-        <is>
-          <t>id_unidad</t>
-        </is>
-      </c>
-      <c r="E18" s="25" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="F18" s="26" t="inlineStr">
-        <is>
-          <t>Historial de cotizaciones por unidad</t>
         </is>
       </c>
     </row>
@@ -6200,12 +6206,12 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>idx_cotizacion_broker</t>
+          <t>idx_cotizacion_unidad</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>nombre_broker, fecha_generacion DESC</t>
+          <t>id_unidad</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -6215,7 +6221,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Historial de cotizaciones por broker</t>
+          <t>Historial de cotizaciones por unidad</t>
         </is>
       </c>
     </row>
@@ -6230,20 +6236,50 @@
       </c>
       <c r="C20" s="26" t="inlineStr">
         <is>
+          <t>idx_cotizacion_broker</t>
+        </is>
+      </c>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>nombre_broker, fecha_generacion DESC</t>
+        </is>
+      </c>
+      <c r="E20" s="25" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr">
+        <is>
+          <t>Historial de cotizaciones por broker</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>cotizacion</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
           <t>idx_cotizacion_fecha</t>
         </is>
       </c>
-      <c r="D20" s="26" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>fecha_generacion DESC</t>
         </is>
       </c>
-      <c r="E20" s="25" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="F20" s="26" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Historial cronológico</t>
         </is>
@@ -6302,7 +6338,7 @@
       </c>
     </row>
     <row r="3" ht="28" customHeight="1">
-      <c r="A3" s="57" t="n">
+      <c r="A3" s="59" t="n">
         <v>1</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -6310,19 +6346,19 @@
           <t>inmobiliaria</t>
         </is>
       </c>
-      <c r="C3" s="58" t="inlineStr">
+      <c r="C3" s="60" t="inlineStr">
         <is>
           <t>chk_inmobiliaria_activo</t>
         </is>
       </c>
-      <c r="D3" s="58" t="inlineStr">
+      <c r="D3" s="60" t="inlineStr">
         <is>
           <t>activo IN (0, 1)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="59" t="n">
+      <c r="A4" s="61" t="n">
         <v>2</v>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -6330,19 +6366,19 @@
           <t>proyecto</t>
         </is>
       </c>
-      <c r="C4" s="60" t="inlineStr">
+      <c r="C4" s="62" t="inlineStr">
         <is>
           <t>chk_proyecto_tipo_entrega</t>
         </is>
       </c>
-      <c r="D4" s="60" t="inlineStr">
+      <c r="D4" s="62" t="inlineStr">
         <is>
           <t>tipo_entrega IN ('Entrega Inmediata', 'Entrega Futura')</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="57" t="n">
+      <c r="A5" s="59" t="n">
         <v>3</v>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -6350,19 +6386,19 @@
           <t>proyecto</t>
         </is>
       </c>
-      <c r="C5" s="58" t="inlineStr">
+      <c r="C5" s="60" t="inlineStr">
         <is>
           <t>chk_proyecto_activo</t>
         </is>
       </c>
-      <c r="D5" s="58" t="inlineStr">
+      <c r="D5" s="60" t="inlineStr">
         <is>
           <t>activo IN (0, 1)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="59" t="n">
+      <c r="A6" s="61" t="n">
         <v>4</v>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -6370,19 +6406,19 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="C6" s="60" t="inlineStr">
+      <c r="C6" s="62" t="inlineStr">
         <is>
           <t>chk_unidad_tipo</t>
         </is>
       </c>
-      <c r="D6" s="60" t="inlineStr">
+      <c r="D6" s="62" t="inlineStr">
         <is>
           <t>tipo_unidad IN ('Departamento', 'Estacionamiento', 'Bodega', 'Local Comercial', 'Local comercial', 'Local', 'Estacionamiento Moto', 'Estacionamiento Comercial', 'Estacionamiento local')</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="57" t="n">
+      <c r="A7" s="59" t="n">
         <v>5</v>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -6390,19 +6426,19 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="C7" s="58" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>chk_unidad_estado</t>
         </is>
       </c>
-      <c r="D7" s="58" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>estado_stock IN ('Disponible', 'Arrendado', 'En Recolocación', 'Reservado')</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="59" t="n">
+      <c r="A8" s="61" t="n">
         <v>6</v>
       </c>
       <c r="B8" s="12" t="inlineStr">
@@ -6410,19 +6446,19 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="C8" s="60" t="inlineStr">
+      <c r="C8" s="62" t="inlineStr">
         <is>
           <t>chk_unidad_precio</t>
         </is>
       </c>
-      <c r="D8" s="60" t="inlineStr">
+      <c r="D8" s="62" t="inlineStr">
         <is>
           <t>precio_lista_uf &gt; 0</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="57" t="n">
+      <c r="A9" s="59" t="n">
         <v>7</v>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -6430,19 +6466,19 @@
           <t>unidad</t>
         </is>
       </c>
-      <c r="C9" s="58" t="inlineStr">
+      <c r="C9" s="60" t="inlineStr">
         <is>
           <t>chk_unidad_sup</t>
         </is>
       </c>
-      <c r="D9" s="58" t="inlineStr">
+      <c r="D9" s="60" t="inlineStr">
         <is>
           <t>superficie_total_m2 &gt;= 0</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="59" t="n">
+      <c r="A10" s="61" t="n">
         <v>8</v>
       </c>
       <c r="B10" s="14" t="inlineStr">
@@ -6450,19 +6486,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C10" s="60" t="inlineStr">
+      <c r="C10" s="62" t="inlineStr">
         <is>
           <t>chk_condicion_reserva</t>
         </is>
       </c>
-      <c r="D10" s="60" t="inlineStr">
+      <c r="D10" s="62" t="inlineStr">
         <is>
           <t>reserva_clp &gt;= 0</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="57" t="n">
+      <c r="A11" s="59" t="n">
         <v>9</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
@@ -6470,19 +6506,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C11" s="58" t="inlineStr">
+      <c r="C11" s="60" t="inlineStr">
         <is>
           <t>chk_condicion_descuento</t>
         </is>
       </c>
-      <c r="D11" s="58" t="inlineStr">
+      <c r="D11" s="60" t="inlineStr">
         <is>
           <t>descuento &gt;= 0 AND descuento &lt;= 1</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="59" t="n">
+      <c r="A12" s="61" t="n">
         <v>10</v>
       </c>
       <c r="B12" s="14" t="inlineStr">
@@ -6490,19 +6526,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C12" s="62" t="inlineStr">
         <is>
           <t>chk_condicion_bono_pie</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr">
+      <c r="D12" s="62" t="inlineStr">
         <is>
           <t>bono_pie &gt;= 0 AND bono_pie &lt;= 1</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="57" t="n">
+      <c r="A13" s="59" t="n">
         <v>11</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
@@ -6510,19 +6546,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C13" s="58" t="inlineStr">
+      <c r="C13" s="60" t="inlineStr">
         <is>
           <t>chk_condicion_cuotas</t>
         </is>
       </c>
-      <c r="D13" s="58" t="inlineStr">
+      <c r="D13" s="60" t="inlineStr">
         <is>
           <t>cuotas_pie &gt;= 0</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="59" t="n">
+      <c r="A14" s="61" t="n">
         <v>12</v>
       </c>
       <c r="B14" s="14" t="inlineStr">
@@ -6530,19 +6566,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C14" s="60" t="inlineStr">
+      <c r="C14" s="62" t="inlineStr">
         <is>
           <t>chk_condicion_pie_constr</t>
         </is>
       </c>
-      <c r="D14" s="60" t="inlineStr">
+      <c r="D14" s="62" t="inlineStr">
         <is>
           <t>pie_periodo_construccion &gt;= 0 AND pie_periodo_construccion &lt;= 1</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
-      <c r="A15" s="57" t="n">
+      <c r="A15" s="59" t="n">
         <v>13</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -6550,19 +6586,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C15" s="58" t="inlineStr">
+      <c r="C15" s="60" t="inlineStr">
         <is>
           <t>chk_condicion_cuoton</t>
         </is>
       </c>
-      <c r="D15" s="58" t="inlineStr">
+      <c r="D15" s="60" t="inlineStr">
         <is>
           <t>cuoton &gt;= 0 AND cuoton &lt;= 1</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="59" t="n">
+      <c r="A16" s="61" t="n">
         <v>14</v>
       </c>
       <c r="B16" s="14" t="inlineStr">
@@ -6570,19 +6606,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C16" s="60" t="inlineStr">
+      <c r="C16" s="62" t="inlineStr">
         <is>
           <t>chk_condicion_cred_dir</t>
         </is>
       </c>
-      <c r="D16" s="60" t="inlineStr">
+      <c r="D16" s="62" t="inlineStr">
         <is>
           <t>pie_credito_directo &gt;= 0 AND pie_credito_directo &lt;= 1</t>
         </is>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="57" t="n">
+      <c r="A17" s="59" t="n">
         <v>15</v>
       </c>
       <c r="B17" s="14" t="inlineStr">
@@ -6590,19 +6626,19 @@
           <t>condicion_comercial</t>
         </is>
       </c>
-      <c r="C17" s="58" t="inlineStr">
+      <c r="C17" s="60" t="inlineStr">
         <is>
           <t>chk_condicion_activo</t>
         </is>
       </c>
-      <c r="D17" s="58" t="inlineStr">
+      <c r="D17" s="60" t="inlineStr">
         <is>
           <t>activo IN (0, 1)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="59" t="n">
+      <c r="A18" s="61" t="n">
         <v>16</v>
       </c>
       <c r="B18" s="17" t="inlineStr">
@@ -6610,19 +6646,19 @@
           <t>bien_conjunto</t>
         </is>
       </c>
-      <c r="C18" s="60" t="inlineStr">
+      <c r="C18" s="62" t="inlineStr">
         <is>
           <t>chk_bc_distintos</t>
         </is>
       </c>
-      <c r="D18" s="60" t="inlineStr">
+      <c r="D18" s="62" t="inlineStr">
         <is>
           <t>id_unidad_principal != id_unidad_asociada</t>
         </is>
       </c>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="57" t="n">
+      <c r="A19" s="59" t="n">
         <v>17</v>
       </c>
       <c r="B19" s="19" t="inlineStr">
@@ -6630,19 +6666,19 @@
           <t>uf_valor</t>
         </is>
       </c>
-      <c r="C19" s="58" t="inlineStr">
+      <c r="C19" s="60" t="inlineStr">
         <is>
           <t>chk_uf_valor</t>
         </is>
       </c>
-      <c r="D19" s="58" t="inlineStr">
+      <c r="D19" s="60" t="inlineStr">
         <is>
           <t>valor_uf &gt; 0</t>
         </is>
       </c>
     </row>
     <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="59" t="n">
+      <c r="A20" s="61" t="n">
         <v>18</v>
       </c>
       <c r="B20" s="22" t="inlineStr">
@@ -6650,19 +6686,19 @@
           <t>parametro_cotizador</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="62" t="inlineStr">
         <is>
           <t>chk_param_categoria</t>
         </is>
       </c>
-      <c r="D20" s="60" t="inlineStr">
+      <c r="D20" s="62" t="inlineStr">
         <is>
           <t>categoria IN ('CAE', 'PIE_PCT', 'PLAZO', 'CONSTANTE')</t>
         </is>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="57" t="n">
+      <c r="A21" s="59" t="n">
         <v>19</v>
       </c>
       <c r="B21" s="22" t="inlineStr">
@@ -6670,19 +6706,19 @@
           <t>parametro_cotizador</t>
         </is>
       </c>
-      <c r="C21" s="58" t="inlineStr">
+      <c r="C21" s="60" t="inlineStr">
         <is>
           <t>chk_param_default</t>
         </is>
       </c>
-      <c r="D21" s="58" t="inlineStr">
+      <c r="D21" s="60" t="inlineStr">
         <is>
           <t>es_default IN (0, 1)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="59" t="n">
+      <c r="A22" s="61" t="n">
         <v>20</v>
       </c>
       <c r="B22" s="22" t="inlineStr">
@@ -6690,12 +6726,12 @@
           <t>parametro_cotizador</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="62" t="inlineStr">
         <is>
           <t>chk_param_activo</t>
         </is>
       </c>
-      <c r="D22" s="60" t="inlineStr">
+      <c r="D22" s="62" t="inlineStr">
         <is>
           <t>activo IN (0, 1)</t>
         </is>
@@ -6779,7 +6815,7 @@
           <t>cae_035</t>
         </is>
       </c>
-      <c r="D3" s="61" t="n">
+      <c r="D3" s="63" t="n">
         <v>0.035</v>
       </c>
       <c r="E3" s="46" t="inlineStr">
@@ -6807,7 +6843,7 @@
           <t>cae_040</t>
         </is>
       </c>
-      <c r="D4" s="61" t="n">
+      <c r="D4" s="63" t="n">
         <v>0.04</v>
       </c>
       <c r="E4" s="46" t="inlineStr">
@@ -6835,7 +6871,7 @@
           <t>cae_045</t>
         </is>
       </c>
-      <c r="D5" s="61" t="n">
+      <c r="D5" s="63" t="n">
         <v>0.045</v>
       </c>
       <c r="E5" s="46" t="inlineStr">
@@ -6863,7 +6899,7 @@
           <t>cae_050</t>
         </is>
       </c>
-      <c r="D6" s="61" t="n">
+      <c r="D6" s="63" t="n">
         <v>0.05</v>
       </c>
       <c r="E6" s="46" t="inlineStr">
@@ -6891,7 +6927,7 @@
           <t>pie_000</t>
         </is>
       </c>
-      <c r="D7" s="62" t="n">
+      <c r="D7" s="64" t="n">
         <v>0</v>
       </c>
       <c r="E7" s="40" t="inlineStr">
@@ -6919,7 +6955,7 @@
           <t>pie_005</t>
         </is>
       </c>
-      <c r="D8" s="62" t="n">
+      <c r="D8" s="64" t="n">
         <v>0.05</v>
       </c>
       <c r="E8" s="40" t="inlineStr">
@@ -6947,7 +6983,7 @@
           <t>pie_010</t>
         </is>
       </c>
-      <c r="D9" s="62" t="n">
+      <c r="D9" s="64" t="n">
         <v>0.1</v>
       </c>
       <c r="E9" s="40" t="inlineStr">
@@ -6975,7 +7011,7 @@
           <t>pie_015</t>
         </is>
       </c>
-      <c r="D10" s="62" t="n">
+      <c r="D10" s="64" t="n">
         <v>0.15</v>
       </c>
       <c r="E10" s="40" t="inlineStr">
@@ -7003,7 +7039,7 @@
           <t>pie_020</t>
         </is>
       </c>
-      <c r="D11" s="62" t="n">
+      <c r="D11" s="64" t="n">
         <v>0.2</v>
       </c>
       <c r="E11" s="40" t="inlineStr">
@@ -7031,7 +7067,7 @@
           <t>pie_025</t>
         </is>
       </c>
-      <c r="D12" s="62" t="n">
+      <c r="D12" s="64" t="n">
         <v>0.25</v>
       </c>
       <c r="E12" s="40" t="inlineStr">
@@ -7059,7 +7095,7 @@
           <t>pie_030</t>
         </is>
       </c>
-      <c r="D13" s="62" t="n">
+      <c r="D13" s="64" t="n">
         <v>0.3</v>
       </c>
       <c r="E13" s="40" t="inlineStr">
@@ -7087,7 +7123,7 @@
           <t>pie_035</t>
         </is>
       </c>
-      <c r="D14" s="62" t="n">
+      <c r="D14" s="64" t="n">
         <v>0.35</v>
       </c>
       <c r="E14" s="40" t="inlineStr">
@@ -7115,7 +7151,7 @@
           <t>pie_040</t>
         </is>
       </c>
-      <c r="D15" s="62" t="n">
+      <c r="D15" s="64" t="n">
         <v>0.4</v>
       </c>
       <c r="E15" s="40" t="inlineStr">
@@ -7143,7 +7179,7 @@
           <t>plazo_20</t>
         </is>
       </c>
-      <c r="D16" s="63" t="n">
+      <c r="D16" s="65" t="n">
         <v>20</v>
       </c>
       <c r="E16" s="38" t="inlineStr">
@@ -7171,7 +7207,7 @@
           <t>plazo_25</t>
         </is>
       </c>
-      <c r="D17" s="63" t="n">
+      <c r="D17" s="65" t="n">
         <v>25</v>
       </c>
       <c r="E17" s="38" t="inlineStr">
@@ -7199,7 +7235,7 @@
           <t>plazo_30</t>
         </is>
       </c>
-      <c r="D18" s="63" t="n">
+      <c r="D18" s="65" t="n">
         <v>30</v>
       </c>
       <c r="E18" s="38" t="inlineStr">
@@ -7214,168 +7250,168 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="59" t="n">
+      <c r="A19" s="61" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="59" t="inlineStr">
+      <c r="B19" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C19" s="60" t="inlineStr">
+      <c r="C19" s="62" t="inlineStr">
         <is>
           <t>UPFRONT_PCT</t>
         </is>
       </c>
-      <c r="D19" s="64" t="n">
+      <c r="D19" s="66" t="n">
         <v>0.02</v>
       </c>
-      <c r="E19" s="60" t="inlineStr">
+      <c r="E19" s="62" t="inlineStr">
         <is>
           <t>Upfront a la Promesa (%)</t>
         </is>
       </c>
-      <c r="F19" s="65" t="inlineStr">
+      <c r="F19" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="59" t="n">
+      <c r="A20" s="61" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="59" t="inlineStr">
+      <c r="B20" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C20" s="60" t="inlineStr">
+      <c r="C20" s="62" t="inlineStr">
         <is>
           <t>APORTE_INMOB_PCT</t>
         </is>
       </c>
-      <c r="D20" s="64" t="n">
+      <c r="D20" s="66" t="n">
         <v>0.1</v>
       </c>
-      <c r="E20" s="60" t="inlineStr">
+      <c r="E20" s="62" t="inlineStr">
         <is>
           <t>Aporte Inmobiliaria (%)</t>
         </is>
       </c>
-      <c r="F20" s="65" t="inlineStr">
+      <c r="F20" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="59" t="n">
+      <c r="A21" s="61" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="59" t="inlineStr">
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C21" s="60" t="inlineStr">
+      <c r="C21" s="62" t="inlineStr">
         <is>
           <t>MESES_ARRIENDO_ANIO</t>
         </is>
       </c>
-      <c r="D21" s="64" t="n">
+      <c r="D21" s="66" t="n">
         <v>11</v>
       </c>
-      <c r="E21" s="60" t="inlineStr">
+      <c r="E21" s="62" t="inlineStr">
         <is>
           <t>Meses de arriendo por año</t>
         </is>
       </c>
-      <c r="F21" s="65" t="inlineStr">
+      <c r="F21" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="59" t="n">
+      <c r="A22" s="61" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="59" t="inlineStr">
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C22" s="60" t="inlineStr">
+      <c r="C22" s="62" t="inlineStr">
         <is>
           <t>HAIRCUT_VENTA</t>
         </is>
       </c>
-      <c r="D22" s="64" t="n">
+      <c r="D22" s="66" t="n">
         <v>0.95</v>
       </c>
-      <c r="E22" s="60" t="inlineStr">
+      <c r="E22" s="62" t="inlineStr">
         <is>
           <t>Factor precio venta año 5</t>
         </is>
       </c>
-      <c r="F22" s="65" t="inlineStr">
+      <c r="F22" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="59" t="n">
+      <c r="A23" s="61" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="59" t="inlineStr">
+      <c r="B23" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C23" s="60" t="inlineStr">
+      <c r="C23" s="62" t="inlineStr">
         <is>
           <t>FACTOR_LTV</t>
         </is>
       </c>
-      <c r="D23" s="64" t="n">
+      <c r="D23" s="66" t="n">
         <v>0.67</v>
       </c>
-      <c r="E23" s="60" t="inlineStr">
+      <c r="E23" s="62" t="inlineStr">
         <is>
           <t>Factor LTV amortización 60 meses</t>
         </is>
       </c>
-      <c r="F23" s="65" t="inlineStr">
+      <c r="F23" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="59" t="n">
+      <c r="A24" s="61" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="59" t="inlineStr">
+      <c r="B24" s="61" t="inlineStr">
         <is>
           <t>CONSTANTE</t>
         </is>
       </c>
-      <c r="C24" s="60" t="inlineStr">
+      <c r="C24" s="62" t="inlineStr">
         <is>
           <t>PLUSVALIA_DEFAULT</t>
         </is>
       </c>
-      <c r="D24" s="64" t="n">
+      <c r="D24" s="66" t="n">
         <v>0.02</v>
       </c>
-      <c r="E24" s="60" t="inlineStr">
+      <c r="E24" s="62" t="inlineStr">
         <is>
           <t>Plusvalía anual estimada default</t>
         </is>
       </c>
-      <c r="F24" s="65" t="inlineStr">
+      <c r="F24" s="67" t="inlineStr">
         <is>
           <t>—</t>
         </is>

</xml_diff>

<commit_message>
Actualiza proyecto base de datos inicial es en excel MODELO_DATOS_COTIZADOR.xlsx, de futuro será en POSTGRESQL. tambien considerar REACT 19
</commit_message>
<xml_diff>
--- a/MODELO_DATOS_COTIZADOR.xlsx
+++ b/MODELO_DATOS_COTIZADOR.xlsx
@@ -34,7 +34,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -862,7 +862,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MODELO DE DATOS — COTIZADOR WEB MERCADO PRIMARIO</t>
+          <t>MODELO DE DATOS — COTIZADOR WEB MERCADO PRIMARIO  |  React 19 + Next.js 15  |  SQLite (dev) → PostgreSQL (prod)</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="C11" s="25" t="inlineStr">
         <is>
-          <t>SQLite</t>
+          <t>SQLite/PG</t>
         </is>
       </c>
       <c r="D11" s="25" t="inlineStr">

</xml_diff>